<commit_message>
Ajout des id transaction iti (#74)
* add iti numbers

* update menu

* update titles

* update workflows 8ad0175d1e88a9fa24da6d64599a2da17b747559
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
+++ b/main/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4214" uniqueCount="770">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4211" uniqueCount="765">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-10-31T16:33:35+00:00</t>
+    <t>2025-04-24T12:56:51+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2005,10 +2005,6 @@
     <t>DocumentReference.context.related.reference</t>
   </si>
   <si>
-    <t>ele-1
-ref-1</t>
-  </si>
-  <si>
     <t>DocumentReference.context.related:referenceIdList.type</t>
   </si>
   <si>
@@ -2208,9 +2204,6 @@
   </si>
   <si>
     <t>A symbol in syntax defined by the system. The symbol may be a predefined code or an expression in a syntax defined by the coding system (e.g. post-coordination).</t>
-  </si>
-  <si>
-    <t>Note that FHIR strings SHALL NOT exceed 1MB in size</t>
   </si>
   <si>
     <t>Need to refer to a particular code in the system.</t>
@@ -2373,17 +2366,9 @@
     <t>Time period during which identifier is/was valid for use.</t>
   </si>
   <si>
-    <t>A Period specifies a range of time; the context of use will specify whether the entire range applies (e.g. "the patient was an inpatient of the hospital for this time range") or one value from the range applies (e.g. "give to the patient between these two times").
-Period is not used for a duration (a measure of elapsed time). See [Duration](http://hl7.org/fhir/R4/datatypes.html#Duration).</t>
-  </si>
-  <si>
     <t>Identifier.period</t>
   </si>
   <si>
-    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-per-1:If present, start SHALL have a lower value than end {start.hasValue().not() or end.hasValue().not() or (start &lt;= end)}</t>
-  </si>
-  <si>
     <t>Role.effectiveTime or implied by context</t>
   </si>
   <si>
@@ -2406,10 +2391,6 @@
   </si>
   <si>
     <t>Identifier.assigner</t>
-  </si>
-  <si>
-    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-ref-1:SHALL have a contained resource if a local reference is provided {reference.startsWith('#').not() or (reference.substring(1).trace('url') in %rootResource.contained.id.trace('ids'))}</t>
   </si>
   <si>
     <t>II.assigningAuthorityName but note that this is an improper use by the definition of the field.  Also Role.scoper</t>
@@ -2741,17 +2722,17 @@
   <dimension ref="A1:AS102"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="81.62109375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="67.2578125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="14.7890625" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="4" max="4" width="39.9140625" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="5" max="5" width="6.77734375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="4.9453125" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="5.4296875" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="16.27734375" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="13.26171875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="69.97265625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="57.66015625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="12.6796875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="4" max="4" width="34.21875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="4.65625" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="180.21875" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="154.50390625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -2760,31 +2741,31 @@
     <col min="17" max="17" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="18" max="18" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="19" max="19" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="20" max="20" width="38.2265625" customWidth="true" bestFit="true"/>
-    <col min="21" max="21" width="17.171875" customWidth="true" bestFit="true"/>
-    <col min="22" max="22" width="17.65625" customWidth="true" bestFit="true"/>
-    <col min="23" max="23" width="19.03515625" customWidth="true" bestFit="true"/>
-    <col min="24" max="24" width="18.859375" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="98.61328125" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="120.0625" customWidth="true" bestFit="true"/>
-    <col min="27" max="27" width="6.34765625" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="22.71875" customWidth="true" bestFit="true"/>
-    <col min="29" max="29" width="43.88671875" customWidth="true" bestFit="true"/>
-    <col min="30" max="30" width="17.21484375" customWidth="true" bestFit="true"/>
-    <col min="31" max="31" width="14.4140625" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="44.0703125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="33" max="33" width="10.5546875" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="34" max="34" width="11.0390625" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" width="32.7734375" customWidth="true" bestFit="true"/>
+    <col min="21" max="21" width="14.72265625" customWidth="true" bestFit="true"/>
+    <col min="22" max="22" width="15.13671875" customWidth="true" bestFit="true"/>
+    <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
+    <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="84.54296875" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="102.93359375" customWidth="true" bestFit="true"/>
+    <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
+    <col min="29" max="29" width="37.625" customWidth="true" bestFit="true"/>
+    <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
+    <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="37.78125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
-    <col min="37" max="37" width="90.72265625" customWidth="true" bestFit="true"/>
-    <col min="38" max="38" width="29.69921875" customWidth="true" bestFit="true"/>
-    <col min="39" max="39" width="52.0078125" customWidth="true" bestFit="true"/>
+    <col min="37" max="37" width="77.77734375" customWidth="true" bestFit="true"/>
+    <col min="38" max="38" width="25.4609375" customWidth="true" bestFit="true"/>
+    <col min="39" max="39" width="44.5859375" customWidth="true" bestFit="true"/>
     <col min="40" max="40" width="255.0" customWidth="true" bestFit="true"/>
     <col min="41" max="41" width="255.0" customWidth="true" bestFit="true"/>
-    <col min="42" max="42" width="36.91796875" customWidth="true" bestFit="true"/>
-    <col min="43" max="43" width="84.2265625" customWidth="true" bestFit="true"/>
-    <col min="44" max="44" width="162.44921875" customWidth="true" bestFit="true"/>
-    <col min="45" max="45" width="80.15625" customWidth="true" bestFit="true"/>
+    <col min="42" max="42" width="31.65234375" customWidth="true" bestFit="true"/>
+    <col min="43" max="43" width="72.20703125" customWidth="true" bestFit="true"/>
+    <col min="44" max="44" width="139.26953125" customWidth="true" bestFit="true"/>
+    <col min="45" max="45" width="68.71875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12923,7 +12904,7 @@
         <v>84</v>
       </c>
       <c r="AI79" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ79" t="s" s="2">
         <v>126</v>
@@ -12938,7 +12919,7 @@
         <v>82</v>
       </c>
       <c r="AN79" t="s" s="2">
-        <v>198</v>
+        <v>115</v>
       </c>
       <c r="AO79" t="s" s="2">
         <v>82</v>
@@ -13052,7 +13033,7 @@
         <v>97</v>
       </c>
       <c r="AI80" t="s" s="2">
-        <v>632</v>
+        <v>590</v>
       </c>
       <c r="AJ80" t="s" s="2">
         <v>109</v>
@@ -13087,10 +13068,10 @@
     </row>
     <row r="81" hidden="true">
       <c r="A81" t="s" s="2">
+        <v>632</v>
+      </c>
+      <c r="B81" t="s" s="2">
         <v>633</v>
-      </c>
-      <c r="B81" t="s" s="2">
-        <v>634</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -13181,7 +13162,7 @@
         <v>97</v>
       </c>
       <c r="AI81" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ81" t="s" s="2">
         <v>109</v>
@@ -13216,10 +13197,10 @@
     </row>
     <row r="82" hidden="true">
       <c r="A82" t="s" s="2">
+        <v>634</v>
+      </c>
+      <c r="B82" t="s" s="2">
         <v>635</v>
-      </c>
-      <c r="B82" t="s" s="2">
-        <v>636</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -13310,7 +13291,7 @@
         <v>97</v>
       </c>
       <c r="AI82" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ82" t="s" s="2">
         <v>109</v>
@@ -13334,7 +13315,7 @@
         <v>82</v>
       </c>
       <c r="AQ82" t="s" s="2">
-        <v>220</v>
+        <v>82</v>
       </c>
       <c r="AR82" t="s" s="2">
         <v>82</v>
@@ -13345,10 +13326,10 @@
     </row>
     <row r="83" hidden="true">
       <c r="A83" t="s" s="2">
+        <v>636</v>
+      </c>
+      <c r="B83" t="s" s="2">
         <v>637</v>
-      </c>
-      <c r="B83" t="s" s="2">
-        <v>638</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -13472,10 +13453,10 @@
     </row>
     <row r="84" hidden="true">
       <c r="A84" t="s" s="2">
+        <v>638</v>
+      </c>
+      <c r="B84" t="s" s="2">
         <v>639</v>
-      </c>
-      <c r="B84" t="s" s="2">
-        <v>640</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -13566,7 +13547,7 @@
         <v>84</v>
       </c>
       <c r="AI84" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ84" t="s" s="2">
         <v>126</v>
@@ -13581,7 +13562,7 @@
         <v>82</v>
       </c>
       <c r="AN84" t="s" s="2">
-        <v>198</v>
+        <v>115</v>
       </c>
       <c r="AO84" t="s" s="2">
         <v>82</v>
@@ -13601,10 +13582,10 @@
     </row>
     <row r="85" hidden="true">
       <c r="A85" t="s" s="2">
+        <v>640</v>
+      </c>
+      <c r="B85" t="s" s="2">
         <v>641</v>
-      </c>
-      <c r="B85" t="s" s="2">
-        <v>642</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -13630,16 +13611,16 @@
         <v>175</v>
       </c>
       <c r="L85" t="s" s="2">
+        <v>642</v>
+      </c>
+      <c r="M85" t="s" s="2">
         <v>643</v>
       </c>
-      <c r="M85" t="s" s="2">
+      <c r="N85" t="s" s="2">
         <v>644</v>
       </c>
-      <c r="N85" t="s" s="2">
+      <c r="O85" t="s" s="2">
         <v>645</v>
-      </c>
-      <c r="O85" t="s" s="2">
-        <v>646</v>
       </c>
       <c r="P85" t="s" s="2">
         <v>82</v>
@@ -13667,29 +13648,29 @@
         <v>241</v>
       </c>
       <c r="Y85" t="s" s="2">
+        <v>646</v>
+      </c>
+      <c r="Z85" t="s" s="2">
         <v>647</v>
       </c>
-      <c r="Z85" t="s" s="2">
+      <c r="AA85" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB85" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC85" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD85" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE85" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF85" t="s" s="2">
         <v>648</v>
       </c>
-      <c r="AA85" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB85" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC85" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD85" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE85" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF85" t="s" s="2">
-        <v>649</v>
-      </c>
       <c r="AG85" t="s" s="2">
         <v>83</v>
       </c>
@@ -13697,7 +13678,7 @@
         <v>97</v>
       </c>
       <c r="AI85" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ85" t="s" s="2">
         <v>109</v>
@@ -13712,7 +13693,7 @@
         <v>82</v>
       </c>
       <c r="AN85" t="s" s="2">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="AO85" t="s" s="2">
         <v>82</v>
@@ -13732,10 +13713,10 @@
     </row>
     <row r="86" hidden="true">
       <c r="A86" t="s" s="2">
+        <v>650</v>
+      </c>
+      <c r="B86" t="s" s="2">
         <v>651</v>
-      </c>
-      <c r="B86" t="s" s="2">
-        <v>652</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -13761,16 +13742,16 @@
         <v>258</v>
       </c>
       <c r="L86" t="s" s="2">
+        <v>652</v>
+      </c>
+      <c r="M86" t="s" s="2">
         <v>653</v>
       </c>
-      <c r="M86" t="s" s="2">
+      <c r="N86" t="s" s="2">
         <v>654</v>
       </c>
-      <c r="N86" t="s" s="2">
+      <c r="O86" t="s" s="2">
         <v>655</v>
-      </c>
-      <c r="O86" t="s" s="2">
-        <v>656</v>
       </c>
       <c r="P86" t="s" s="2">
         <v>82</v>
@@ -13798,29 +13779,29 @@
         <v>157</v>
       </c>
       <c r="Y86" t="s" s="2">
+        <v>656</v>
+      </c>
+      <c r="Z86" t="s" s="2">
         <v>657</v>
       </c>
-      <c r="Z86" t="s" s="2">
+      <c r="AA86" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB86" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC86" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD86" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE86" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF86" t="s" s="2">
         <v>658</v>
       </c>
-      <c r="AA86" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB86" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC86" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD86" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE86" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF86" t="s" s="2">
-        <v>659</v>
-      </c>
       <c r="AG86" t="s" s="2">
         <v>83</v>
       </c>
@@ -13828,7 +13809,7 @@
         <v>97</v>
       </c>
       <c r="AI86" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ86" t="s" s="2">
         <v>109</v>
@@ -13843,7 +13824,7 @@
         <v>82</v>
       </c>
       <c r="AN86" t="s" s="2">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="AO86" t="s" s="2">
         <v>82</v>
@@ -13852,7 +13833,7 @@
         <v>82</v>
       </c>
       <c r="AQ86" t="s" s="2">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="AR86" t="s" s="2">
         <v>82</v>
@@ -13863,10 +13844,10 @@
     </row>
     <row r="87" hidden="true">
       <c r="A87" t="s" s="2">
+        <v>660</v>
+      </c>
+      <c r="B87" t="s" s="2">
         <v>661</v>
-      </c>
-      <c r="B87" t="s" s="2">
-        <v>662</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -13990,10 +13971,10 @@
     </row>
     <row r="88" hidden="true">
       <c r="A88" t="s" s="2">
+        <v>662</v>
+      </c>
+      <c r="B88" t="s" s="2">
         <v>663</v>
-      </c>
-      <c r="B88" t="s" s="2">
-        <v>664</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -14084,7 +14065,7 @@
         <v>84</v>
       </c>
       <c r="AI88" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ88" t="s" s="2">
         <v>126</v>
@@ -14099,7 +14080,7 @@
         <v>82</v>
       </c>
       <c r="AN88" t="s" s="2">
-        <v>198</v>
+        <v>115</v>
       </c>
       <c r="AO88" t="s" s="2">
         <v>82</v>
@@ -14119,10 +14100,10 @@
     </row>
     <row r="89" hidden="true">
       <c r="A89" t="s" s="2">
+        <v>664</v>
+      </c>
+      <c r="B89" t="s" s="2">
         <v>665</v>
-      </c>
-      <c r="B89" t="s" s="2">
-        <v>666</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -14148,16 +14129,16 @@
         <v>153</v>
       </c>
       <c r="L89" t="s" s="2">
+        <v>666</v>
+      </c>
+      <c r="M89" t="s" s="2">
         <v>667</v>
       </c>
-      <c r="M89" t="s" s="2">
+      <c r="N89" t="s" s="2">
         <v>668</v>
       </c>
-      <c r="N89" t="s" s="2">
+      <c r="O89" t="s" s="2">
         <v>669</v>
-      </c>
-      <c r="O89" t="s" s="2">
-        <v>670</v>
       </c>
       <c r="P89" t="s" s="2">
         <v>82</v>
@@ -14206,7 +14187,7 @@
         <v>82</v>
       </c>
       <c r="AF89" t="s" s="2">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="AG89" t="s" s="2">
         <v>83</v>
@@ -14215,7 +14196,7 @@
         <v>84</v>
       </c>
       <c r="AI89" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ89" t="s" s="2">
         <v>109</v>
@@ -14230,16 +14211,16 @@
         <v>82</v>
       </c>
       <c r="AN89" t="s" s="2">
+        <v>671</v>
+      </c>
+      <c r="AO89" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AP89" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ89" t="s" s="2">
         <v>672</v>
-      </c>
-      <c r="AO89" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP89" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ89" t="s" s="2">
-        <v>673</v>
       </c>
       <c r="AR89" t="s" s="2">
         <v>82</v>
@@ -14250,10 +14231,10 @@
     </row>
     <row r="90" hidden="true">
       <c r="A90" t="s" s="2">
+        <v>673</v>
+      </c>
+      <c r="B90" t="s" s="2">
         <v>674</v>
-      </c>
-      <c r="B90" t="s" s="2">
-        <v>675</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -14377,10 +14358,10 @@
     </row>
     <row r="91" hidden="true">
       <c r="A91" t="s" s="2">
+        <v>675</v>
+      </c>
+      <c r="B91" t="s" s="2">
         <v>676</v>
-      </c>
-      <c r="B91" t="s" s="2">
-        <v>677</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -14471,7 +14452,7 @@
         <v>84</v>
       </c>
       <c r="AI91" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ91" t="s" s="2">
         <v>126</v>
@@ -14486,7 +14467,7 @@
         <v>82</v>
       </c>
       <c r="AN91" t="s" s="2">
-        <v>198</v>
+        <v>115</v>
       </c>
       <c r="AO91" t="s" s="2">
         <v>82</v>
@@ -14506,10 +14487,10 @@
     </row>
     <row r="92" hidden="true">
       <c r="A92" t="s" s="2">
+        <v>677</v>
+      </c>
+      <c r="B92" t="s" s="2">
         <v>678</v>
-      </c>
-      <c r="B92" t="s" s="2">
-        <v>679</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -14535,16 +14516,16 @@
         <v>140</v>
       </c>
       <c r="L92" t="s" s="2">
+        <v>679</v>
+      </c>
+      <c r="M92" t="s" s="2">
         <v>680</v>
       </c>
-      <c r="M92" t="s" s="2">
+      <c r="N92" t="s" s="2">
         <v>681</v>
       </c>
-      <c r="N92" t="s" s="2">
+      <c r="O92" t="s" s="2">
         <v>682</v>
-      </c>
-      <c r="O92" t="s" s="2">
-        <v>683</v>
       </c>
       <c r="P92" t="s" s="2">
         <v>82</v>
@@ -14554,47 +14535,47 @@
         <v>82</v>
       </c>
       <c r="S92" t="s" s="2">
+        <v>683</v>
+      </c>
+      <c r="T92" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U92" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V92" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W92" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X92" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y92" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z92" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA92" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB92" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC92" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD92" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE92" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF92" t="s" s="2">
         <v>684</v>
       </c>
-      <c r="T92" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U92" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V92" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W92" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X92" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y92" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z92" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA92" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB92" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC92" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD92" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE92" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF92" t="s" s="2">
-        <v>685</v>
-      </c>
       <c r="AG92" t="s" s="2">
         <v>83</v>
       </c>
@@ -14602,7 +14583,7 @@
         <v>97</v>
       </c>
       <c r="AI92" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ92" t="s" s="2">
         <v>109</v>
@@ -14617,16 +14598,16 @@
         <v>82</v>
       </c>
       <c r="AN92" t="s" s="2">
+        <v>685</v>
+      </c>
+      <c r="AO92" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AP92" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ92" t="s" s="2">
         <v>686</v>
-      </c>
-      <c r="AO92" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP92" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ92" t="s" s="2">
-        <v>687</v>
       </c>
       <c r="AR92" t="s" s="2">
         <v>82</v>
@@ -14637,10 +14618,10 @@
     </row>
     <row r="93" hidden="true">
       <c r="A93" t="s" s="2">
+        <v>687</v>
+      </c>
+      <c r="B93" t="s" s="2">
         <v>688</v>
-      </c>
-      <c r="B93" t="s" s="2">
-        <v>689</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -14666,13 +14647,13 @@
         <v>111</v>
       </c>
       <c r="L93" t="s" s="2">
+        <v>689</v>
+      </c>
+      <c r="M93" t="s" s="2">
         <v>690</v>
       </c>
-      <c r="M93" t="s" s="2">
+      <c r="N93" t="s" s="2">
         <v>691</v>
-      </c>
-      <c r="N93" t="s" s="2">
-        <v>692</v>
       </c>
       <c r="O93" s="2"/>
       <c r="P93" t="s" s="2">
@@ -14722,7 +14703,7 @@
         <v>82</v>
       </c>
       <c r="AF93" t="s" s="2">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="AG93" t="s" s="2">
         <v>83</v>
@@ -14731,7 +14712,7 @@
         <v>97</v>
       </c>
       <c r="AI93" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ93" t="s" s="2">
         <v>109</v>
@@ -14746,16 +14727,16 @@
         <v>82</v>
       </c>
       <c r="AN93" t="s" s="2">
+        <v>693</v>
+      </c>
+      <c r="AO93" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AP93" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ93" t="s" s="2">
         <v>694</v>
-      </c>
-      <c r="AO93" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP93" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ93" t="s" s="2">
-        <v>695</v>
       </c>
       <c r="AR93" t="s" s="2">
         <v>82</v>
@@ -14766,10 +14747,10 @@
     </row>
     <row r="94" hidden="true">
       <c r="A94" t="s" s="2">
+        <v>695</v>
+      </c>
+      <c r="B94" t="s" s="2">
         <v>696</v>
-      </c>
-      <c r="B94" t="s" s="2">
-        <v>697</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
@@ -14795,16 +14776,14 @@
         <v>175</v>
       </c>
       <c r="L94" t="s" s="2">
+        <v>697</v>
+      </c>
+      <c r="M94" t="s" s="2">
         <v>698</v>
       </c>
-      <c r="M94" t="s" s="2">
+      <c r="N94" s="2"/>
+      <c r="O94" t="s" s="2">
         <v>699</v>
-      </c>
-      <c r="N94" t="s" s="2">
-        <v>700</v>
-      </c>
-      <c r="O94" t="s" s="2">
-        <v>701</v>
       </c>
       <c r="P94" t="s" s="2">
         <v>82</v>
@@ -14853,7 +14832,7 @@
         <v>82</v>
       </c>
       <c r="AF94" t="s" s="2">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>83</v>
@@ -14862,7 +14841,7 @@
         <v>97</v>
       </c>
       <c r="AI94" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ94" t="s" s="2">
         <v>109</v>
@@ -14886,7 +14865,7 @@
         <v>82</v>
       </c>
       <c r="AQ94" t="s" s="2">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="AR94" t="s" s="2">
         <v>82</v>
@@ -14897,10 +14876,10 @@
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -14926,16 +14905,14 @@
         <v>111</v>
       </c>
       <c r="L95" t="s" s="2">
+        <v>704</v>
+      </c>
+      <c r="M95" t="s" s="2">
+        <v>705</v>
+      </c>
+      <c r="N95" s="2"/>
+      <c r="O95" t="s" s="2">
         <v>706</v>
-      </c>
-      <c r="M95" t="s" s="2">
-        <v>707</v>
-      </c>
-      <c r="N95" t="s" s="2">
-        <v>700</v>
-      </c>
-      <c r="O95" t="s" s="2">
-        <v>708</v>
       </c>
       <c r="P95" t="s" s="2">
         <v>82</v>
@@ -14984,7 +14961,7 @@
         <v>82</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>83</v>
@@ -14993,7 +14970,7 @@
         <v>97</v>
       </c>
       <c r="AI95" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ95" t="s" s="2">
         <v>109</v>
@@ -15008,7 +14985,7 @@
         <v>82</v>
       </c>
       <c r="AN95" t="s" s="2">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="AO95" t="s" s="2">
         <v>82</v>
@@ -15017,7 +14994,7 @@
         <v>82</v>
       </c>
       <c r="AQ95" t="s" s="2">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="AR95" t="s" s="2">
         <v>82</v>
@@ -15028,10 +15005,10 @@
     </row>
     <row r="96" hidden="true">
       <c r="A96" t="s" s="2">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -15054,19 +15031,19 @@
         <v>98</v>
       </c>
       <c r="K96" t="s" s="2">
+        <v>712</v>
+      </c>
+      <c r="L96" t="s" s="2">
+        <v>713</v>
+      </c>
+      <c r="M96" t="s" s="2">
         <v>714</v>
       </c>
-      <c r="L96" t="s" s="2">
+      <c r="N96" t="s" s="2">
         <v>715</v>
       </c>
-      <c r="M96" t="s" s="2">
+      <c r="O96" t="s" s="2">
         <v>716</v>
-      </c>
-      <c r="N96" t="s" s="2">
-        <v>717</v>
-      </c>
-      <c r="O96" t="s" s="2">
-        <v>718</v>
       </c>
       <c r="P96" t="s" s="2">
         <v>82</v>
@@ -15115,7 +15092,7 @@
         <v>82</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>83</v>
@@ -15124,7 +15101,7 @@
         <v>97</v>
       </c>
       <c r="AI96" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ96" t="s" s="2">
         <v>109</v>
@@ -15139,7 +15116,7 @@
         <v>82</v>
       </c>
       <c r="AN96" t="s" s="2">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="AO96" t="s" s="2">
         <v>82</v>
@@ -15148,7 +15125,7 @@
         <v>82</v>
       </c>
       <c r="AQ96" t="s" s="2">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="AR96" t="s" s="2">
         <v>82</v>
@@ -15159,10 +15136,10 @@
     </row>
     <row r="97" hidden="true">
       <c r="A97" t="s" s="2">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -15188,16 +15165,16 @@
         <v>111</v>
       </c>
       <c r="L97" t="s" s="2">
+        <v>722</v>
+      </c>
+      <c r="M97" t="s" s="2">
+        <v>723</v>
+      </c>
+      <c r="N97" t="s" s="2">
         <v>724</v>
       </c>
-      <c r="M97" t="s" s="2">
+      <c r="O97" t="s" s="2">
         <v>725</v>
-      </c>
-      <c r="N97" t="s" s="2">
-        <v>726</v>
-      </c>
-      <c r="O97" t="s" s="2">
-        <v>727</v>
       </c>
       <c r="P97" t="s" s="2">
         <v>82</v>
@@ -15246,7 +15223,7 @@
         <v>82</v>
       </c>
       <c r="AF97" t="s" s="2">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="AG97" t="s" s="2">
         <v>83</v>
@@ -15255,7 +15232,7 @@
         <v>97</v>
       </c>
       <c r="AI97" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ97" t="s" s="2">
         <v>109</v>
@@ -15270,7 +15247,7 @@
         <v>82</v>
       </c>
       <c r="AN97" t="s" s="2">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="AO97" t="s" s="2">
         <v>82</v>
@@ -15279,7 +15256,7 @@
         <v>82</v>
       </c>
       <c r="AQ97" t="s" s="2">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="AR97" t="s" s="2">
         <v>82</v>
@@ -15290,10 +15267,10 @@
     </row>
     <row r="98" hidden="true">
       <c r="A98" t="s" s="2">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -15319,16 +15296,16 @@
         <v>140</v>
       </c>
       <c r="L98" t="s" s="2">
+        <v>731</v>
+      </c>
+      <c r="M98" t="s" s="2">
+        <v>732</v>
+      </c>
+      <c r="N98" t="s" s="2">
         <v>733</v>
       </c>
-      <c r="M98" t="s" s="2">
+      <c r="O98" t="s" s="2">
         <v>734</v>
-      </c>
-      <c r="N98" t="s" s="2">
-        <v>735</v>
-      </c>
-      <c r="O98" t="s" s="2">
-        <v>736</v>
       </c>
       <c r="P98" t="s" s="2">
         <v>82</v>
@@ -15341,7 +15318,7 @@
         <v>82</v>
       </c>
       <c r="T98" t="s" s="2">
-        <v>737</v>
+        <v>735</v>
       </c>
       <c r="U98" t="s" s="2">
         <v>82</v>
@@ -15377,7 +15354,7 @@
         <v>82</v>
       </c>
       <c r="AF98" t="s" s="2">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="AG98" t="s" s="2">
         <v>83</v>
@@ -15386,7 +15363,7 @@
         <v>97</v>
       </c>
       <c r="AI98" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ98" t="s" s="2">
         <v>109</v>
@@ -15401,7 +15378,7 @@
         <v>82</v>
       </c>
       <c r="AN98" t="s" s="2">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="AO98" t="s" s="2">
         <v>82</v>
@@ -15410,7 +15387,7 @@
         <v>82</v>
       </c>
       <c r="AQ98" t="s" s="2">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="AR98" t="s" s="2">
         <v>82</v>
@@ -15421,10 +15398,10 @@
     </row>
     <row r="99" hidden="true">
       <c r="A99" t="s" s="2">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -15450,13 +15427,13 @@
         <v>111</v>
       </c>
       <c r="L99" t="s" s="2">
+        <v>741</v>
+      </c>
+      <c r="M99" t="s" s="2">
+        <v>742</v>
+      </c>
+      <c r="N99" t="s" s="2">
         <v>743</v>
-      </c>
-      <c r="M99" t="s" s="2">
-        <v>744</v>
-      </c>
-      <c r="N99" t="s" s="2">
-        <v>745</v>
       </c>
       <c r="O99" s="2"/>
       <c r="P99" t="s" s="2">
@@ -15470,7 +15447,7 @@
         <v>82</v>
       </c>
       <c r="T99" t="s" s="2">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="U99" t="s" s="2">
         <v>82</v>
@@ -15506,7 +15483,7 @@
         <v>82</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>83</v>
@@ -15515,7 +15492,7 @@
         <v>97</v>
       </c>
       <c r="AI99" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ99" t="s" s="2">
         <v>109</v>
@@ -15530,7 +15507,7 @@
         <v>82</v>
       </c>
       <c r="AN99" t="s" s="2">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="AO99" t="s" s="2">
         <v>82</v>
@@ -15539,7 +15516,7 @@
         <v>82</v>
       </c>
       <c r="AQ99" t="s" s="2">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="AR99" t="s" s="2">
         <v>82</v>
@@ -15550,10 +15527,10 @@
     </row>
     <row r="100" hidden="true">
       <c r="A100" t="s" s="2">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -15579,14 +15556,12 @@
         <v>531</v>
       </c>
       <c r="L100" t="s" s="2">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="M100" t="s" s="2">
-        <v>753</v>
-      </c>
-      <c r="N100" t="s" s="2">
-        <v>754</v>
-      </c>
+        <v>751</v>
+      </c>
+      <c r="N100" s="2"/>
       <c r="O100" s="2"/>
       <c r="P100" t="s" s="2">
         <v>82</v>
@@ -15635,7 +15610,7 @@
         <v>82</v>
       </c>
       <c r="AF100" t="s" s="2">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>83</v>
@@ -15644,10 +15619,10 @@
         <v>97</v>
       </c>
       <c r="AI100" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ100" t="s" s="2">
-        <v>756</v>
+        <v>109</v>
       </c>
       <c r="AK100" t="s" s="2">
         <v>82</v>
@@ -15659,7 +15634,7 @@
         <v>82</v>
       </c>
       <c r="AN100" t="s" s="2">
-        <v>757</v>
+        <v>753</v>
       </c>
       <c r="AO100" t="s" s="2">
         <v>82</v>
@@ -15668,7 +15643,7 @@
         <v>82</v>
       </c>
       <c r="AQ100" t="s" s="2">
-        <v>758</v>
+        <v>754</v>
       </c>
       <c r="AR100" t="s" s="2">
         <v>82</v>
@@ -15679,10 +15654,10 @@
     </row>
     <row r="101" hidden="true">
       <c r="A101" t="s" s="2">
-        <v>759</v>
+        <v>755</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>760</v>
+        <v>756</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -15708,13 +15683,13 @@
         <v>332</v>
       </c>
       <c r="L101" t="s" s="2">
-        <v>761</v>
+        <v>757</v>
       </c>
       <c r="M101" t="s" s="2">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="N101" t="s" s="2">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="O101" s="2"/>
       <c r="P101" t="s" s="2">
@@ -15764,7 +15739,7 @@
         <v>82</v>
       </c>
       <c r="AF101" t="s" s="2">
-        <v>764</v>
+        <v>760</v>
       </c>
       <c r="AG101" t="s" s="2">
         <v>83</v>
@@ -15773,10 +15748,10 @@
         <v>97</v>
       </c>
       <c r="AI101" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ101" t="s" s="2">
-        <v>765</v>
+        <v>109</v>
       </c>
       <c r="AK101" t="s" s="2">
         <v>82</v>
@@ -15788,7 +15763,7 @@
         <v>82</v>
       </c>
       <c r="AN101" t="s" s="2">
-        <v>766</v>
+        <v>761</v>
       </c>
       <c r="AO101" t="s" s="2">
         <v>82</v>
@@ -15797,7 +15772,7 @@
         <v>82</v>
       </c>
       <c r="AQ101" t="s" s="2">
-        <v>767</v>
+        <v>762</v>
       </c>
       <c r="AR101" t="s" s="2">
         <v>82</v>
@@ -15808,10 +15783,10 @@
     </row>
     <row r="102" hidden="true">
       <c r="A102" t="s" s="2">
-        <v>768</v>
+        <v>763</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>769</v>
+        <v>764</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -15902,7 +15877,7 @@
         <v>97</v>
       </c>
       <c r="AI102" t="s" s="2">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="AJ102" t="s" s="2">
         <v>109</v>

</xml_diff>

<commit_message>
rm TRE A04 (#72) f86d09ebaa90a497eea04f6137c435a71bfaee07
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
+++ b/main/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-04-24T12:56:51+00:00</t>
+    <t>2025-04-24T12:57:11+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -838,7 +838,7 @@
     <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
 constr-bind-type:Les valeurs possibles pour cet élément doivent provenir d’une des terminologies de référence suivantes :
  TRE_A05-TypeDocComplementaireCISIS, OID : 1.2.250.1.213.1.1.4.12
- TRE_A04-TypeDocument-LOINC, OID : 2.16.840.1.113883.6.1
+ LOINC, OID : 2.16.840.1.113883.6.1
  TRE_A12-NomenclatureASTM, OID : ASTM
 Les valeurs possibles peuvent être restreintes en fonction du jeu de valeurs correspondant mis à disposition par le projet (exemple : JDV_J66-TypeCode-DMP).
 En l’absence de spécifications complémentaires, le jeu de valeurs JDV_J07-XdsTypeCode-CISIS peut être utilisé. {null}</t>

</xml_diff>

<commit_message>
Revise authenticator min cardinality : make it optional (#89)
* Revise authenticator cardinality : make it optional

Updated the authenticator attribute description for clarity.

* Update authenticator description in FSH profile

* Update PDSm_ComprehensiveDocumentReference.fsh

* align simplifiedpublish et comprehensivedocumentreference

* update 7069880a4da58ef9c66bb4aecb3894881f052522
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
+++ b/main/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-06T07:19:11+00:00</t>
+    <t>2026-05-27T14:14:06+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -988,7 +988,7 @@
     <t>DocumentReference.author</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/fhir/annuaire/StructureDefinition/as-practitionerrole|Device|https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-patient) &lt;&lt;contained&gt;&gt;
+    <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/fhir/annuaire/StructureDefinition/as-practitioner|https://interop.esante.gouv.fr/ig/fhir/annuaire/StructureDefinition/as-practitionerrole|Device|https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-patient) &lt;&lt;contained&gt;&gt;
 </t>
   </si>
   <si>
@@ -1025,11 +1025,11 @@
     <t>DocumentReference.authenticator</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/fhir/annuaire/StructureDefinition/as-practitionerrole|https://interop.esante.gouv.fr/ig/fhir/annuaire/StructureDefinition/as-organization) &lt;&lt;contained&gt;&gt;
+    <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/fhir/annuaire/StructureDefinition/as-practitioner|https://interop.esante.gouv.fr/ig/fhir/annuaire/StructureDefinition/as-practitionerrole|https://interop.esante.gouv.fr/ig/fhir/annuaire/StructureDefinition/as-organization) &lt;&lt;contained&gt;&gt;
 </t>
   </si>
   <si>
-    <t>Cet attribut représente l’acteur validant le document et prenant la responsabilité du contenu médical de celui-ci. Il peut s’agir de l’auteur du document si celui-ci est une personne et s’il endosse la responsabilité du contenu médical de ses documents. Si l’auteur est un dispositif, cet attribut doit représenter la personne responsable de l’action effectuée par le dispositif. Pour les documents d’expression personnelle du patient, cet attribut fait référence au patient.</t>
+    <t>Cet attribut représente l’acteur validant le document et prenant la responsabilité du contenu médical de celui-ci. Il peut s’agir de l’auteur du document si celui-ci est une personne et s’il endosse la responsabilité du contenu médical de ses documents.</t>
   </si>
   <si>
     <t>Which person or organization authenticates that this document is valid.</t>
@@ -2735,7 +2735,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="154.50390625" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="218.3359375" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -6513,7 +6513,7 @@
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="G30" t="s" s="2">
         <v>97</v>

</xml_diff>

<commit_message>
feat: adopt container mode for CI-build workflow (#118)
* feat: adopt container mode for CI-build workflow

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>

* Rename workflow for CI-build on GitHub pages

* Update fhir-workflows.yml

---------

Co-authored-by: Claude Sonnet 4.6 <noreply@anthropic.com> 5961e773d7341638e24bbb7fd97f41627bedd8fe
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
+++ b/main/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-03T13:50:50+00:00</t>
+    <t>2026-06-30T13:26:19+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1207,7 +1207,7 @@
     <t>DocumentReference.description</t>
   </si>
   <si>
-    <t>Commentaire associé au document.</t>
+    <t>Description du document source, lisible par l'homme, correspondant au commentaire associé au document</t>
   </si>
   <si>
     <t>Human-readable description of the source document.</t>

</xml_diff>